<commit_message>
F-4: unassigned asset cost. Support-asset cost not assigned to a working unit is spread evenly across the units with a red banner; an unassigned productive asset blocks.
Scenario A and A misaligned 217 of 217 live. Expected script A-7, calc map s7, Cost Allocation brief Addendum 2, stress brief Addendum 19.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SGr6C5GL21exfbPdJ1tWVd
</commit_message>
<xml_diff>
--- a/docs/fin_mirra_v6.1/Audit/v6_0/smoke_test/3.1 Stress Test/scenario_a/review_scenario_a.xlsx
+++ b/docs/fin_mirra_v6.1/Audit/v6_0/smoke_test/3.1 Stress Test/scenario_a/review_scenario_a.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Staff" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Groups" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PnL" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rate_Builder" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Staff" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Assets" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Groups" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="PnL" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Rate_Builder" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of 2026-10-17. Values are computed by mirra_expected.py (independent of the app). Read-only record - change the recipe, not this file.</t>
+          <t>As of 2026-10-25. Values are computed by mirra_expected.py (independent of the app). Read-only record - change the recipe, not this file.</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>812167.28</v>
+        <v>804077.75</v>
       </c>
     </row>
     <row r="6">
@@ -510,7 +510,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>41829.83</v>
+        <v>41530.97</v>
       </c>
     </row>
     <row r="8">
@@ -530,7 +530,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>41829.83</v>
+        <v>41530.97</v>
       </c>
     </row>
     <row r="10">
@@ -560,7 +560,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>812167.28</v>
+        <v>804077.75</v>
       </c>
     </row>
     <row r="13">
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>41829.83</v>
+        <v>41530.97</v>
       </c>
     </row>
     <row r="14">
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>1015707.81</v>
+        <v>1007319.41</v>
       </c>
     </row>
     <row r="16">
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>1015707.81</v>
+        <v>1007319.41</v>
       </c>
     </row>
     <row r="19">
@@ -650,7 +650,7 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>102.61</v>
+        <v>101.76</v>
       </c>
     </row>
     <row r="22">
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>9414.83</v>
+        <v>9321.549999999999</v>
       </c>
     </row>
     <row r="34">
@@ -780,7 +780,7 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>9414.83</v>
+        <v>9321.549999999999</v>
       </c>
     </row>
     <row r="35">
@@ -894,7 +894,7 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>812167.28</v>
+        <v>804077.75</v>
       </c>
     </row>
     <row r="47">
@@ -904,7 +904,7 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>41829.83</v>
+        <v>41530.97</v>
       </c>
     </row>
     <row r="48">
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>129742.86</v>
+        <v>138131.26</v>
       </c>
     </row>
     <row r="49">
@@ -1108,7 +1108,7 @@
         <v>1011.3</v>
       </c>
       <c r="N2" s="5" t="n">
-        <v>74949.06</v>
+        <v>74206.5</v>
       </c>
     </row>
     <row r="3">
@@ -1158,7 +1158,7 @@
         <v>1011.3</v>
       </c>
       <c r="N3" s="5" t="n">
-        <v>74949.06</v>
+        <v>74206.5</v>
       </c>
     </row>
     <row r="4">
@@ -1208,7 +1208,7 @@
         <v>1011.3</v>
       </c>
       <c r="N4" s="5" t="n">
-        <v>74949.06</v>
+        <v>74206.5</v>
       </c>
     </row>
     <row r="5">
@@ -1258,7 +1258,7 @@
         <v>1011.3</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>74949.06</v>
+        <v>74206.5</v>
       </c>
     </row>
     <row r="6">
@@ -1308,7 +1308,7 @@
         <v>1189.76</v>
       </c>
       <c r="N6" s="5" t="n">
-        <v>88175.36</v>
+        <v>87301.75999999999</v>
       </c>
     </row>
     <row r="7">
@@ -1358,7 +1358,7 @@
         <v>1189.76</v>
       </c>
       <c r="N7" s="5" t="n">
-        <v>88175.36</v>
+        <v>87301.75999999999</v>
       </c>
     </row>
     <row r="8">
@@ -1408,7 +1408,7 @@
         <v>1368.22</v>
       </c>
       <c r="N8" s="5" t="n">
-        <v>101502.13</v>
+        <v>100397.02</v>
       </c>
     </row>
     <row r="9">
@@ -1458,7 +1458,7 @@
         <v>91.52</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>119816.84</v>
+        <v>118495.52</v>
       </c>
     </row>
     <row r="10">
@@ -1508,7 +1508,7 @@
         <v>49.92</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>65289.12</v>
+        <v>64633.92</v>
       </c>
     </row>
     <row r="11">
@@ -1558,7 +1558,7 @@
         <v>37.94</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>49412.25</v>
+        <v>49121.78</v>
       </c>
     </row>
   </sheetData>
@@ -1702,10 +1702,10 @@
         <v>1680</v>
       </c>
       <c r="L2" s="5" t="n">
-        <v>15551.33</v>
+        <v>15452.77</v>
       </c>
       <c r="M2" s="5" t="n">
-        <v>9.2567</v>
+        <v>9.1981</v>
       </c>
     </row>
     <row r="3">
@@ -1753,10 +1753,10 @@
         <v>1440</v>
       </c>
       <c r="L3" s="5" t="n">
-        <v>5357.25</v>
+        <v>5313.88</v>
       </c>
       <c r="M3" s="5" t="n">
-        <v>3.7203</v>
+        <v>3.6902</v>
       </c>
     </row>
     <row r="4">
@@ -1804,10 +1804,10 @@
         <v>1680</v>
       </c>
       <c r="L4" s="5" t="n">
-        <v>12820.29</v>
+        <v>12749.32</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>7.6311</v>
+        <v>7.5889</v>
       </c>
     </row>
     <row r="5">
@@ -1855,10 +1855,10 @@
         <v>1225</v>
       </c>
       <c r="L5" s="5" t="n">
-        <v>1872.69</v>
+        <v>1833.26</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>1.5287</v>
+        <v>1.4965</v>
       </c>
     </row>
     <row r="6">
@@ -1906,7 +1906,7 @@
         <v>0</v>
       </c>
       <c r="L6" s="5" t="n">
-        <v>2532.95</v>
+        <v>2508.75</v>
       </c>
       <c r="M6" s="5" t="n">
         <v>0</v>
@@ -1957,7 +1957,7 @@
         <v>0</v>
       </c>
       <c r="L7" s="5" t="n">
-        <v>3695.32</v>
+        <v>3672.98</v>
       </c>
       <c r="M7" s="5" t="n">
         <v>0</v>
@@ -2382,7 +2382,7 @@
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>35010.98</v>
+        <v>26921.44</v>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
@@ -2712,7 +2712,7 @@
         </is>
       </c>
       <c r="E16" s="5" t="n">
-        <v>41829.83</v>
+        <v>41530.97</v>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>

</xml_diff>